<commit_message>
Apunta datos del vídeo 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LGV9XSbx6L88nquaNrvjoA
</commit_message>
<xml_diff>
--- a/seguimiento-videos-catboing.xlsx
+++ b/seguimiento-videos-catboing.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="69">
   <si>
     <t xml:space="preserve">Nº</t>
   </si>
@@ -172,6 +172,24 @@
     <t xml:space="preserve">Se frenó a las 2 h (~620) y luego casi plano. 43 % México. Subido solo 4 h después del vídeo 2. Abandono máximo en el seg. 1.</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mi gato a las 3 AM 😩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Humor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mujer dormida y gato tocándole la cara (noche, oscuro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historia problema→solución + "Comenta GATO". Mejor retención (62 %, 10 s: 10,4 %) pero se frenó en ~350 a la 1 h. Primer fotograma oscuro.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen de vídeos Catboing</t>
   </si>
   <si>
@@ -215,9 +233,6 @@
   </si>
   <si>
     <t xml:space="preserve">% pasa seg. 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Humor</t>
   </si>
   <si>
     <t xml:space="preserve">Tensión</t>
@@ -1013,28 +1028,62 @@
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="6" t="str">
+      <c r="H5" s="4" t="n">
+        <v>367</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>265</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <f aca="false">IF(OR(H5="",H5=0),"",J5/H5)</f>
-        <v/>
-      </c>
-      <c r="L5" s="7"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="5"/>
+        <v>0.389645776566758</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
@@ -5022,57 +5071,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B3" s="10" t="n">
         <f aca="false">COUNT(Videos!$H$2:$H$151)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">SUM(Videos!$H$2:$H$151)</f>
-        <v>1646</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">IFERROR(AVERAGE(Videos!$H$2:$H$151),"")</f>
-        <v>548.666666666667</v>
+        <v>503.25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">IFERROR(SUM(Videos!$J$2:$J$151)/SUM(Videos!$H$2:$H$151),"")</f>
-        <v>0.381530984204131</v>
+        <v>0.38301043219076</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">SUM(Videos!$Q$2:$Q$151)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B8" s="10" t="n">
         <f aca="false">SUM(Videos!$R$2:$R$151)</f>
@@ -5081,7 +5130,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(Videos!$S$2:$S$151)</f>
@@ -5090,7 +5139,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">IFERROR(INDEX(Videos!$A$2:$A$151,MATCH(MAX(Videos!$H$2:$H$151),Videos!$H$2:$H$151,0)),"")</f>
@@ -5099,7 +5148,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(INDEX(Videos!$A$2:$A$151,MATCH(MAX(Videos!$K$2:$K$151),Videos!$K$2:$K$151,0)),"")</f>
@@ -5108,21 +5157,21 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5144,24 +5193,24 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">COUNTIFS(Videos!$E$2:$E$151,A16,Videos!$H$2:$H$151,"&gt;0")</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="15" t="str">
+        <v>1</v>
+      </c>
+      <c r="C16" s="15" t="n">
         <f aca="false">IFERROR(AVERAGEIFS(Videos!$H$2:$H$151,Videos!$E$2:$E$151,A16),"")</f>
-        <v/>
-      </c>
-      <c r="D16" s="16" t="str">
+        <v>367</v>
+      </c>
+      <c r="D16" s="16" t="n">
         <f aca="false">IFERROR(SUMIFS(Videos!$J$2:$J$151,Videos!$E$2:$E$151,A16)/SUMIFS(Videos!$H$2:$H$151,Videos!$E$2:$E$151,A16),"")</f>
-        <v/>
+        <v>0.389645776566758</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">COUNTIFS(Videos!$E$2:$E$151,A17,Videos!$H$2:$H$151,"&gt;0")</f>
@@ -5195,7 +5244,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">COUNTIFS(Videos!$E$2:$E$151,A19,Videos!$H$2:$H$151,"&gt;0")</f>
@@ -5234,42 +5283,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="18" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>